<commit_message>
Checking push from other pc
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results.xlsx
+++ b/rss_islandr/templates/results.xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{46F99A3F-4744-4F77-B1F1-37D7A89DCEF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
   <si>
     <t>Soil</t>
   </si>
@@ -122,21 +136,12 @@
   </si>
   <si>
     <t>Industrial</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Pathological waste and animal carcasses</t>
-  </si>
-  <si>
-    <t>Small</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -681,8 +686,68 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="31" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -693,66 +758,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -776,9 +781,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -816,9 +821,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -853,7 +858,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -888,7 +893,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1061,7 +1066,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1069,32 +1074,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="31"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="2">
-        <v>158568</v>
-      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -1109,10 +1112,10 @@
       <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1147,31 +1150,31 @@
       <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="29"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="31"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="37"/>
+      <c r="B6" s="35"/>
       <c r="C6" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1187,12 +1190,12 @@
       <c r="O6" s="6"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="18" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1208,12 +1211,12 @@
       <c r="O7" s="7"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="18" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1229,12 +1232,12 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="35"/>
+      <c r="B9" s="37"/>
       <c r="C9" s="5">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1250,237 +1253,237 @@
       <c r="O9" s="9"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="31"/>
     </row>
     <row r="11" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="24" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="24" t="s">
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="25"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="24" t="s">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="25"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="24" t="s">
+      <c r="K11" s="23"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="25"/>
-      <c r="O11" s="26"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="24"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="31"/>
+      <c r="B12" s="33"/>
       <c r="C12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="31"/>
+      <c r="E12" s="33"/>
       <c r="F12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="G12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="31"/>
+      <c r="H12" s="33"/>
       <c r="I12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="J12" s="30" t="s">
+      <c r="J12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="K12" s="31"/>
+      <c r="K12" s="33"/>
       <c r="L12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="30" t="s">
+      <c r="M12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="N12" s="31"/>
+      <c r="N12" s="33"/>
       <c r="O12" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="33"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="33"/>
+      <c r="E13" s="28"/>
       <c r="F13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="33"/>
+      <c r="H13" s="28"/>
       <c r="I13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="36" t="s">
+      <c r="J13" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="37"/>
+      <c r="K13" s="35"/>
       <c r="L13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="36" t="s">
+      <c r="M13" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="N13" s="37"/>
+      <c r="N13" s="35"/>
       <c r="O13" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="33"/>
+      <c r="E14" s="28"/>
       <c r="F14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="33"/>
+      <c r="H14" s="28"/>
       <c r="I14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J14" s="36" t="s">
+      <c r="J14" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="37"/>
+      <c r="K14" s="35"/>
       <c r="L14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M14" s="36" t="s">
+      <c r="M14" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="N14" s="37"/>
+      <c r="N14" s="35"/>
       <c r="O14" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="33"/>
+      <c r="E15" s="28"/>
       <c r="F15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="G15" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="35"/>
+      <c r="H15" s="37"/>
       <c r="I15" s="11">
         <v>0</v>
       </c>
-      <c r="J15" s="36" t="s">
+      <c r="J15" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="K15" s="37"/>
+      <c r="K15" s="35"/>
       <c r="L15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="36" t="s">
+      <c r="M15" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="37"/>
+      <c r="N15" s="35"/>
       <c r="O15" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="21"/>
+      <c r="B16" s="41"/>
       <c r="C16" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="35"/>
+      <c r="E16" s="37"/>
       <c r="F16" s="11">
         <v>0</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="34" t="s">
+      <c r="J16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="35"/>
+      <c r="K16" s="37"/>
       <c r="L16" s="11">
         <v>0</v>
       </c>
-      <c r="M16" s="34" t="s">
+      <c r="M16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="N16" s="35"/>
+      <c r="N16" s="37"/>
       <c r="O16" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="23"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="10">
         <v>0</v>
       </c>
@@ -1498,174 +1501,209 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="28"/>
-      <c r="M18" s="28"/>
-      <c r="N18" s="28"/>
-      <c r="O18" s="29"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="31"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="str">
+      <c r="A19" s="22" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="24" t="str">
+      <c r="B19" s="23"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="22" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="24" t="str">
+      <c r="E19" s="23"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="22" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="25"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="24" t="str">
+      <c r="H19" s="23"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="22" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="25"/>
-      <c r="L19" s="26"/>
-      <c r="M19" s="24" t="str">
+      <c r="K19" s="23"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="22" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="25"/>
-      <c r="O19" s="26"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="41"/>
+      <c r="B20" s="26"/>
       <c r="C20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="41"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="G20" s="40" t="s">
+      <c r="G20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="41"/>
+      <c r="H20" s="26"/>
       <c r="I20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="J20" s="40" t="s">
+      <c r="J20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="K20" s="41"/>
+      <c r="K20" s="26"/>
       <c r="L20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="M20" s="40" t="s">
+      <c r="M20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N20" s="41"/>
+      <c r="N20" s="26"/>
       <c r="O20" s="17" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="28"/>
       <c r="C21" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="33"/>
+      <c r="E21" s="28"/>
       <c r="F21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="32" t="s">
+      <c r="G21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="33"/>
+      <c r="H21" s="28"/>
       <c r="I21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="32" t="s">
+      <c r="J21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="K21" s="33"/>
+      <c r="K21" s="28"/>
       <c r="L21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="M21" s="32" t="s">
+      <c r="M21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="N21" s="33"/>
+      <c r="N21" s="28"/>
       <c r="O21" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="43"/>
+      <c r="B22" s="21"/>
       <c r="C22" s="19">
         <v>0</v>
       </c>
-      <c r="D22" s="42" t="s">
+      <c r="D22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="43"/>
+      <c r="E22" s="21"/>
       <c r="F22" s="19">
         <v>0</v>
       </c>
-      <c r="G22" s="42" t="s">
+      <c r="G22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="43"/>
+      <c r="H22" s="21"/>
       <c r="I22" s="19">
         <v>0</v>
       </c>
-      <c r="J22" s="42" t="s">
+      <c r="J22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="43"/>
+      <c r="K22" s="21"/>
       <c r="L22" s="19">
         <v>0</v>
       </c>
-      <c r="M22" s="42" t="s">
+      <c r="M22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="N22" s="43"/>
+      <c r="N22" s="21"/>
       <c r="O22" s="10">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A20:B20"/>
@@ -1682,46 +1720,11 @@
     <mergeCell ref="M22:N22"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed paths and implemented notebook widget to use in assessment
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results.xlsx
+++ b/rss_islandr/templates/results.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{596C7D69-9D09-4429-811C-417C73EA745D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3120" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
   <si>
     <t>Soil</t>
   </si>
@@ -136,18 +135,12 @@
   </si>
   <si>
     <t>Industrial</t>
-  </si>
-  <si>
-    <t>Airports (NACE Code H.52.23)</t>
-  </si>
-  <si>
-    <t>Artificial Surfaces - Mine, dump and construction sites</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -694,76 +687,76 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -787,9 +780,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -827,9 +820,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -864,7 +857,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -899,7 +892,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1072,7 +1065,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1080,29 +1073,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="31"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="29"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="35"/>
+      <c r="B2" s="37"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -1110,9 +1103,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -1120,10 +1111,10 @@
       <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="28"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1143,9 +1134,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="39"/>
-      <c r="C4" s="4" t="s">
-        <v>36</v>
-      </c>
+      <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -1160,29 +1149,29 @@
       <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="31"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="29"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="35"/>
+      <c r="B6" s="37"/>
       <c r="C6" s="18" t="s">
         <v>32</v>
       </c>
@@ -1200,10 +1189,10 @@
       <c r="O6" s="6"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="18" t="s">
         <v>32</v>
       </c>
@@ -1221,10 +1210,10 @@
       <c r="O7" s="7"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
         <v>32</v>
       </c>
@@ -1242,10 +1231,10 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="37"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="5">
         <v>0</v>
       </c>
@@ -1263,237 +1252,237 @@
       <c r="O9" s="9"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="31"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="28"/>
+      <c r="M10" s="28"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="29"/>
     </row>
     <row r="11" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="22" t="s">
+      <c r="B11" s="25"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22" t="s">
+      <c r="E11" s="25"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="22" t="s">
+      <c r="H11" s="25"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="23"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="22" t="s">
+      <c r="K11" s="25"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="23"/>
-      <c r="O11" s="24"/>
+      <c r="N11" s="25"/>
+      <c r="O11" s="26"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="33"/>
+      <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="33"/>
+      <c r="E12" s="31"/>
       <c r="F12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="33"/>
+      <c r="H12" s="31"/>
       <c r="I12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="J12" s="32" t="s">
+      <c r="J12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="K12" s="33"/>
+      <c r="K12" s="31"/>
       <c r="L12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="32" t="s">
+      <c r="M12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="N12" s="33"/>
+      <c r="N12" s="31"/>
       <c r="O12" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="28"/>
+      <c r="E13" s="33"/>
       <c r="F13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="28"/>
+      <c r="H13" s="33"/>
       <c r="I13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="34" t="s">
+      <c r="J13" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="35"/>
+      <c r="K13" s="37"/>
       <c r="L13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="34" t="s">
+      <c r="M13" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="N13" s="35"/>
+      <c r="N13" s="37"/>
       <c r="O13" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="28"/>
+      <c r="E14" s="33"/>
       <c r="F14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="G14" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="28"/>
+      <c r="H14" s="33"/>
       <c r="I14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J14" s="34" t="s">
+      <c r="J14" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="35"/>
+      <c r="K14" s="37"/>
       <c r="L14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M14" s="34" t="s">
+      <c r="M14" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="N14" s="35"/>
+      <c r="N14" s="37"/>
       <c r="O14" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="D15" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="28"/>
+      <c r="E15" s="33"/>
       <c r="F15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="36" t="s">
+      <c r="G15" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="37"/>
+      <c r="H15" s="35"/>
       <c r="I15" s="11">
         <v>0</v>
       </c>
-      <c r="J15" s="34" t="s">
+      <c r="J15" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="K15" s="35"/>
+      <c r="K15" s="37"/>
       <c r="L15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="34" t="s">
+      <c r="M15" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="35"/>
+      <c r="N15" s="37"/>
       <c r="O15" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="40" t="s">
+      <c r="A16" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="41"/>
+      <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="36" t="s">
+      <c r="D16" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="37"/>
+      <c r="E16" s="35"/>
       <c r="F16" s="11">
         <v>0</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="36" t="s">
+      <c r="J16" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="37"/>
+      <c r="K16" s="35"/>
       <c r="L16" s="11">
         <v>0</v>
       </c>
-      <c r="M16" s="36" t="s">
+      <c r="M16" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="N16" s="37"/>
+      <c r="N16" s="35"/>
       <c r="O16" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="43"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="10">
         <v>0</v>
       </c>
@@ -1511,169 +1500,214 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="31"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
+      <c r="K18" s="28"/>
+      <c r="L18" s="28"/>
+      <c r="M18" s="28"/>
+      <c r="N18" s="28"/>
+      <c r="O18" s="29"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="str">
+      <c r="A19" s="24" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="22" t="str">
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="24" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22" t="str">
+      <c r="E19" s="25"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="24" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22" t="str">
+      <c r="H19" s="25"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="24" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="23"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="22" t="str">
+      <c r="K19" s="25"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="24" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="23"/>
-      <c r="O19" s="24"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="26"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="26"/>
+      <c r="B20" s="41"/>
       <c r="C20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="26"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="G20" s="25" t="s">
+      <c r="G20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="26"/>
+      <c r="H20" s="41"/>
       <c r="I20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="J20" s="25" t="s">
+      <c r="J20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="K20" s="26"/>
+      <c r="K20" s="41"/>
       <c r="L20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="M20" s="25" t="s">
+      <c r="M20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="N20" s="26"/>
+      <c r="N20" s="41"/>
       <c r="O20" s="17" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="28"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="27" t="s">
+      <c r="D21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="28"/>
+      <c r="E21" s="33"/>
       <c r="F21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="27" t="s">
+      <c r="G21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="28"/>
+      <c r="H21" s="33"/>
       <c r="I21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="27" t="s">
+      <c r="J21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="K21" s="28"/>
+      <c r="K21" s="33"/>
       <c r="L21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="M21" s="27" t="s">
+      <c r="M21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="N21" s="28"/>
+      <c r="N21" s="33"/>
       <c r="O21" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="21"/>
+      <c r="B22" s="43"/>
       <c r="C22" s="19">
         <v>0</v>
       </c>
-      <c r="D22" s="20" t="s">
+      <c r="D22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="21"/>
+      <c r="E22" s="43"/>
       <c r="F22" s="19">
         <v>0</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="21"/>
+      <c r="H22" s="43"/>
       <c r="I22" s="19">
         <v>0</v>
       </c>
-      <c r="J22" s="20" t="s">
+      <c r="J22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="21"/>
+      <c r="K22" s="43"/>
       <c r="L22" s="19">
         <v>0</v>
       </c>
-      <c r="M22" s="20" t="s">
+      <c r="M22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="N22" s="21"/>
+      <c r="N22" s="43"/>
       <c r="O22" s="10">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="61">
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="M11:O11"/>
@@ -1690,51 +1724,6 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Need to create interface in AssessNotebookUI
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results.xlsx
+++ b/rss_islandr/templates/results.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="42">
   <si>
     <t>Soil</t>
   </si>
@@ -135,6 +135,24 @@
   </si>
   <si>
     <t>Industrial</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>&lt;1m</t>
+  </si>
+  <si>
+    <t>Bio-accumulative and toxic materials</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>No access</t>
   </si>
 </sst>
 </file>
@@ -687,6 +705,66 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -697,66 +775,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1073,29 +1091,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="31"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="37"/>
+      <c r="B2" s="35"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -1111,10 +1129,10 @@
       <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1149,31 +1167,31 @@
       <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="29"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="31"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="37"/>
+      <c r="B6" s="35"/>
       <c r="C6" s="18" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1189,12 +1207,12 @@
       <c r="O6" s="6"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1210,12 +1228,12 @@
       <c r="O7" s="7"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1231,12 +1249,12 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="35"/>
+      <c r="B9" s="37"/>
       <c r="C9" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1252,239 +1270,239 @@
       <c r="O9" s="9"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="31"/>
     </row>
     <row r="11" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="24" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="24" t="s">
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="25"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="24" t="s">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="25"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="24" t="s">
+      <c r="K11" s="23"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="25"/>
-      <c r="O11" s="26"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="24"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="31"/>
+      <c r="B12" s="33"/>
       <c r="C12" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="31"/>
+      <c r="E12" s="33"/>
       <c r="F12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="G12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="31"/>
+      <c r="H12" s="33"/>
       <c r="I12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="J12" s="30" t="s">
+      <c r="J12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="K12" s="31"/>
+      <c r="K12" s="33"/>
       <c r="L12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="30" t="s">
+      <c r="M12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="N12" s="31"/>
+      <c r="N12" s="33"/>
       <c r="O12" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="33"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="33"/>
+      <c r="E13" s="28"/>
       <c r="F13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="33"/>
+      <c r="H13" s="28"/>
       <c r="I13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="36" t="s">
+      <c r="J13" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="37"/>
+      <c r="K13" s="35"/>
       <c r="L13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="36" t="s">
+      <c r="M13" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="N13" s="37"/>
+      <c r="N13" s="35"/>
       <c r="O13" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="33"/>
+      <c r="E14" s="28"/>
       <c r="F14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="33"/>
+      <c r="H14" s="28"/>
       <c r="I14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J14" s="36" t="s">
+      <c r="J14" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="37"/>
+      <c r="K14" s="35"/>
       <c r="L14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M14" s="36" t="s">
+      <c r="M14" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="N14" s="37"/>
+      <c r="N14" s="35"/>
       <c r="O14" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="33"/>
+      <c r="E15" s="28"/>
       <c r="F15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="G15" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="35"/>
+      <c r="H15" s="37"/>
       <c r="I15" s="11">
         <v>0</v>
       </c>
-      <c r="J15" s="36" t="s">
+      <c r="J15" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="K15" s="37"/>
+      <c r="K15" s="35"/>
       <c r="L15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="36" t="s">
+      <c r="M15" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="37"/>
+      <c r="N15" s="35"/>
       <c r="O15" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="21"/>
+      <c r="B16" s="41"/>
       <c r="C16" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="35"/>
+      <c r="E16" s="37"/>
       <c r="F16" s="11">
         <v>0</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="34" t="s">
+      <c r="J16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="35"/>
+      <c r="K16" s="37"/>
       <c r="L16" s="11">
         <v>0</v>
       </c>
-      <c r="M16" s="34" t="s">
+      <c r="M16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="N16" s="35"/>
+      <c r="N16" s="37"/>
       <c r="O16" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="23"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="10">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1500,174 +1518,209 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="28"/>
-      <c r="M18" s="28"/>
-      <c r="N18" s="28"/>
-      <c r="O18" s="29"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="31"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="str">
+      <c r="A19" s="22" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="24" t="str">
+      <c r="B19" s="23"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="22" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="24" t="str">
+      <c r="E19" s="23"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="22" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="25"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="24" t="str">
+      <c r="H19" s="23"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="22" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="25"/>
-      <c r="L19" s="26"/>
-      <c r="M19" s="24" t="str">
+      <c r="K19" s="23"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="22" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="25"/>
-      <c r="O19" s="26"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="41"/>
+      <c r="B20" s="26"/>
       <c r="C20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="41"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="G20" s="40" t="s">
+      <c r="G20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="41"/>
+      <c r="H20" s="26"/>
       <c r="I20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="J20" s="40" t="s">
+      <c r="J20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="K20" s="41"/>
+      <c r="K20" s="26"/>
       <c r="L20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="M20" s="40" t="s">
+      <c r="M20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N20" s="41"/>
+      <c r="N20" s="26"/>
       <c r="O20" s="17" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="28"/>
       <c r="C21" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="33"/>
+      <c r="E21" s="28"/>
       <c r="F21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="32" t="s">
+      <c r="G21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="33"/>
+      <c r="H21" s="28"/>
       <c r="I21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="32" t="s">
+      <c r="J21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="K21" s="33"/>
+      <c r="K21" s="28"/>
       <c r="L21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="M21" s="32" t="s">
+      <c r="M21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="N21" s="33"/>
+      <c r="N21" s="28"/>
       <c r="O21" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="43"/>
+      <c r="B22" s="21"/>
       <c r="C22" s="19">
-        <v>0</v>
-      </c>
-      <c r="D22" s="42" t="s">
+        <v>0.15</v>
+      </c>
+      <c r="D22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="43"/>
+      <c r="E22" s="21"/>
       <c r="F22" s="19">
         <v>0</v>
       </c>
-      <c r="G22" s="42" t="s">
+      <c r="G22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="43"/>
+      <c r="H22" s="21"/>
       <c r="I22" s="19">
         <v>0</v>
       </c>
-      <c r="J22" s="42" t="s">
+      <c r="J22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="43"/>
+      <c r="K22" s="21"/>
       <c r="L22" s="19">
         <v>0</v>
       </c>
-      <c r="M22" s="42" t="s">
+      <c r="M22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="N22" s="43"/>
+      <c r="N22" s="21"/>
       <c r="O22" s="10">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A20:B20"/>
@@ -1684,46 +1737,11 @@
     <mergeCell ref="M22:N22"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
BUG FIX of notebooks creation. Interfaces probably are not relevant here, but code cleanup should follow
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results.xlsx
+++ b/rss_islandr/templates/results.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{34F173B4-97A4-4424-B440-6E9402067A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3120" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="43">
   <si>
     <t>Soil</t>
   </si>
@@ -137,28 +138,31 @@
     <t>Industrial</t>
   </si>
   <si>
+    <t>Toxic metals</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>&gt;=3m</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>No limit to access</t>
+  </si>
+  <si>
     <t>High</t>
   </si>
   <si>
-    <t>&lt;1m</t>
-  </si>
-  <si>
-    <t>Bio-accumulative and toxic materials</t>
-  </si>
-  <si>
-    <t>Large</t>
-  </si>
-  <si>
     <t>None</t>
-  </si>
-  <si>
-    <t>No access</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -705,76 +709,76 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -798,9 +802,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -838,9 +842,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -875,7 +879,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -910,7 +914,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1083,7 +1087,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1091,29 +1095,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="31"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="29"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="35"/>
+      <c r="B2" s="37"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -1129,10 +1133,10 @@
       <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="28"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1167,31 +1171,31 @@
       <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="31"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="29"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="35"/>
+      <c r="B6" s="37"/>
       <c r="C6" s="18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1207,10 +1211,10 @@
       <c r="O6" s="6"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="28"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="18" t="s">
         <v>39</v>
       </c>
@@ -1228,12 +1232,12 @@
       <c r="O7" s="7"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="28"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1249,12 +1253,12 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="37"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="5">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1270,239 +1274,239 @@
       <c r="O9" s="9"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="31"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="28"/>
+      <c r="M10" s="28"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="29"/>
     </row>
     <row r="11" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="22" t="s">
+      <c r="B11" s="25"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22" t="s">
+      <c r="E11" s="25"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="22" t="s">
+      <c r="H11" s="25"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="23"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="22" t="s">
+      <c r="K11" s="25"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="23"/>
-      <c r="O11" s="24"/>
+      <c r="N11" s="25"/>
+      <c r="O11" s="26"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="33"/>
+      <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="33"/>
+      <c r="E12" s="31"/>
       <c r="F12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="33"/>
+      <c r="H12" s="31"/>
       <c r="I12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="J12" s="32" t="s">
+      <c r="J12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="K12" s="33"/>
+      <c r="K12" s="31"/>
       <c r="L12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="32" t="s">
+      <c r="M12" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="N12" s="33"/>
+      <c r="N12" s="31"/>
       <c r="O12" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="28"/>
+      <c r="E13" s="33"/>
       <c r="F13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="28"/>
+      <c r="H13" s="33"/>
       <c r="I13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="34" t="s">
+      <c r="J13" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="35"/>
+      <c r="K13" s="37"/>
       <c r="L13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="34" t="s">
+      <c r="M13" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="N13" s="35"/>
+      <c r="N13" s="37"/>
       <c r="O13" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="28"/>
+      <c r="E14" s="33"/>
       <c r="F14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="G14" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="28"/>
+      <c r="H14" s="33"/>
       <c r="I14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J14" s="34" t="s">
+      <c r="J14" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="35"/>
+      <c r="K14" s="37"/>
       <c r="L14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M14" s="34" t="s">
+      <c r="M14" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="N14" s="35"/>
+      <c r="N14" s="37"/>
       <c r="O14" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="28"/>
+      <c r="E15" s="33"/>
       <c r="F15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="36" t="s">
+      <c r="G15" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="37"/>
+      <c r="H15" s="35"/>
       <c r="I15" s="11">
         <v>0</v>
       </c>
-      <c r="J15" s="34" t="s">
+      <c r="J15" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="K15" s="35"/>
+      <c r="K15" s="37"/>
       <c r="L15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="34" t="s">
+      <c r="M15" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="35"/>
+      <c r="N15" s="37"/>
       <c r="O15" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="40" t="s">
+      <c r="A16" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="41"/>
+      <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="37"/>
+      <c r="E16" s="35"/>
       <c r="F16" s="11">
         <v>0</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="36" t="s">
+      <c r="J16" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="37"/>
+      <c r="K16" s="35"/>
       <c r="L16" s="11">
         <v>0</v>
       </c>
-      <c r="M16" s="36" t="s">
+      <c r="M16" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="N16" s="37"/>
+      <c r="N16" s="35"/>
       <c r="O16" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="43"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="10">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1518,169 +1522,214 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="31"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
+      <c r="K18" s="28"/>
+      <c r="L18" s="28"/>
+      <c r="M18" s="28"/>
+      <c r="N18" s="28"/>
+      <c r="O18" s="29"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="str">
+      <c r="A19" s="24" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="22" t="str">
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="24" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22" t="str">
+      <c r="E19" s="25"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="24" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22" t="str">
+      <c r="H19" s="25"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="24" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="23"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="22" t="str">
+      <c r="K19" s="25"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="24" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="23"/>
-      <c r="O19" s="24"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="26"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="26"/>
+      <c r="B20" s="41"/>
       <c r="C20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="26"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="G20" s="25" t="s">
+      <c r="G20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="26"/>
+      <c r="H20" s="41"/>
       <c r="I20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="J20" s="25" t="s">
+      <c r="J20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="K20" s="26"/>
+      <c r="K20" s="41"/>
       <c r="L20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="M20" s="25" t="s">
+      <c r="M20" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="N20" s="26"/>
+      <c r="N20" s="41"/>
       <c r="O20" s="17" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="28"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="27" t="s">
+      <c r="D21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="28"/>
+      <c r="E21" s="33"/>
       <c r="F21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="27" t="s">
+      <c r="G21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="28"/>
+      <c r="H21" s="33"/>
       <c r="I21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="27" t="s">
+      <c r="J21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="K21" s="28"/>
+      <c r="K21" s="33"/>
       <c r="L21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="M21" s="27" t="s">
+      <c r="M21" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="N21" s="28"/>
+      <c r="N21" s="33"/>
       <c r="O21" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="21"/>
+      <c r="B22" s="43"/>
       <c r="C22" s="19">
-        <v>0.15</v>
-      </c>
-      <c r="D22" s="20" t="s">
+        <v>2.1951999999999899E-2</v>
+      </c>
+      <c r="D22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="21"/>
+      <c r="E22" s="43"/>
       <c r="F22" s="19">
         <v>0</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="21"/>
+      <c r="H22" s="43"/>
       <c r="I22" s="19">
         <v>0</v>
       </c>
-      <c r="J22" s="20" t="s">
+      <c r="J22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="21"/>
+      <c r="K22" s="43"/>
       <c r="L22" s="19">
         <v>0</v>
       </c>
-      <c r="M22" s="20" t="s">
+      <c r="M22" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="N22" s="21"/>
+      <c r="N22" s="43"/>
       <c r="O22" s="10">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="61">
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="M11:O11"/>
@@ -1697,51 +1746,6 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Code improvements for clarity reasons
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results.xlsx
+++ b/rss_islandr/templates/results.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{34F173B4-97A4-4424-B440-6E9402067A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="44">
   <si>
     <t>Soil</t>
   </si>
@@ -138,31 +137,34 @@
     <t>Industrial</t>
   </si>
   <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>2m</t>
+  </si>
+  <si>
+    <t>This is my site</t>
+  </si>
+  <si>
+    <t>Battery manufacture or recycling</t>
+  </si>
+  <si>
+    <t>Agricultural areas - Permanent crops</t>
+  </si>
+  <si>
     <t>Toxic metals</t>
   </si>
   <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>&gt;=3m</t>
-  </si>
-  <si>
-    <t>Large</t>
-  </si>
-  <si>
     <t>No limit to access</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>None</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -709,6 +711,66 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="32" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="34" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -719,66 +781,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -802,9 +804,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -842,9 +844,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -879,7 +881,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -914,7 +916,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1087,7 +1089,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1095,37 +1097,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="31"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="J2" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -1133,10 +1139,10 @@
       <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="33"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1156,7 +1162,9 @@
         <v>5</v>
       </c>
       <c r="B4" s="39"/>
-      <c r="C4" s="4"/>
+      <c r="C4" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -1171,31 +1179,31 @@
       <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="29"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="31"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="37"/>
+      <c r="B6" s="35"/>
       <c r="C6" s="18" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1211,12 +1219,12 @@
       <c r="O6" s="6"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="18" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1232,10 +1240,10 @@
       <c r="O7" s="7"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="18" t="s">
         <v>37</v>
       </c>
@@ -1253,12 +1261,12 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="35"/>
+      <c r="B9" s="37"/>
       <c r="C9" s="5">
-        <v>0.7</v>
+        <v>0.48999999999999899</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1274,239 +1282,239 @@
       <c r="O9" s="9"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="28"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="29"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="31"/>
     </row>
     <row r="11" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="24" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="25"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="24" t="s">
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="25"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="24" t="s">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="25"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="24" t="s">
+      <c r="K11" s="23"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="25"/>
-      <c r="O11" s="26"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="24"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="31"/>
+      <c r="B12" s="33"/>
       <c r="C12" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="31"/>
+      <c r="E12" s="33"/>
       <c r="F12" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="G12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="31"/>
+      <c r="H12" s="33"/>
       <c r="I12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="J12" s="30" t="s">
+      <c r="J12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="K12" s="31"/>
+      <c r="K12" s="33"/>
       <c r="L12" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="30" t="s">
+      <c r="M12" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="N12" s="31"/>
+      <c r="N12" s="33"/>
       <c r="O12" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="33"/>
+      <c r="B13" s="28"/>
       <c r="C13" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="33"/>
+      <c r="E13" s="28"/>
       <c r="F13" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="33"/>
+      <c r="H13" s="28"/>
       <c r="I13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J13" s="36" t="s">
+      <c r="J13" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="37"/>
+      <c r="K13" s="35"/>
       <c r="L13" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="36" t="s">
+      <c r="M13" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="N13" s="37"/>
+      <c r="N13" s="35"/>
       <c r="O13" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="28"/>
       <c r="C14" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="33"/>
+      <c r="E14" s="28"/>
       <c r="F14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="33"/>
+      <c r="H14" s="28"/>
       <c r="I14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="J14" s="36" t="s">
+      <c r="J14" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="37"/>
+      <c r="K14" s="35"/>
       <c r="L14" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M14" s="36" t="s">
+      <c r="M14" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="N14" s="37"/>
+      <c r="N14" s="35"/>
       <c r="O14" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="33"/>
+      <c r="E15" s="28"/>
       <c r="F15" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="G15" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="H15" s="35"/>
+      <c r="H15" s="37"/>
       <c r="I15" s="11">
         <v>0</v>
       </c>
-      <c r="J15" s="36" t="s">
+      <c r="J15" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="K15" s="37"/>
+      <c r="K15" s="35"/>
       <c r="L15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="36" t="s">
+      <c r="M15" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="37"/>
+      <c r="N15" s="35"/>
       <c r="O15" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="21"/>
+      <c r="B16" s="41"/>
       <c r="C16" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="35"/>
+      <c r="E16" s="37"/>
       <c r="F16" s="11">
         <v>0</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="34" t="s">
+      <c r="J16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="35"/>
+      <c r="K16" s="37"/>
       <c r="L16" s="11">
         <v>0</v>
       </c>
-      <c r="M16" s="34" t="s">
+      <c r="M16" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="N16" s="35"/>
+      <c r="N16" s="37"/>
       <c r="O16" s="11">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="23"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="10">
-        <v>0.4</v>
+        <v>0.44799999999999901</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1522,174 +1530,209 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="23.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="28"/>
-      <c r="M18" s="28"/>
-      <c r="N18" s="28"/>
-      <c r="O18" s="29"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="31"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="str">
+      <c r="A19" s="22" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="24" t="str">
+      <c r="B19" s="23"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="22" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="24" t="str">
+      <c r="E19" s="23"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="22" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="25"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="24" t="str">
+      <c r="H19" s="23"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="22" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="25"/>
-      <c r="L19" s="26"/>
-      <c r="M19" s="24" t="str">
+      <c r="K19" s="23"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="22" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="25"/>
-      <c r="O19" s="26"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="41"/>
+      <c r="B20" s="26"/>
       <c r="C20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="D20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="41"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="G20" s="40" t="s">
+      <c r="G20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="41"/>
+      <c r="H20" s="26"/>
       <c r="I20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="J20" s="40" t="s">
+      <c r="J20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="K20" s="41"/>
+      <c r="K20" s="26"/>
       <c r="L20" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="M20" s="40" t="s">
+      <c r="M20" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N20" s="41"/>
+      <c r="N20" s="26"/>
       <c r="O20" s="17" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="32" t="s">
+      <c r="A21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="28"/>
       <c r="C21" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="33"/>
+      <c r="E21" s="28"/>
       <c r="F21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="32" t="s">
+      <c r="G21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="33"/>
+      <c r="H21" s="28"/>
       <c r="I21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="32" t="s">
+      <c r="J21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="K21" s="33"/>
+      <c r="K21" s="28"/>
       <c r="L21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="M21" s="32" t="s">
+      <c r="M21" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="N21" s="33"/>
+      <c r="N21" s="28"/>
       <c r="O21" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="43"/>
+      <c r="B22" s="21"/>
       <c r="C22" s="19">
-        <v>2.1951999999999899E-2</v>
-      </c>
-      <c r="D22" s="42" t="s">
+        <v>0.109759999999999</v>
+      </c>
+      <c r="D22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="43"/>
+      <c r="E22" s="21"/>
       <c r="F22" s="19">
         <v>0</v>
       </c>
-      <c r="G22" s="42" t="s">
+      <c r="G22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="H22" s="43"/>
+      <c r="H22" s="21"/>
       <c r="I22" s="19">
         <v>0</v>
       </c>
-      <c r="J22" s="42" t="s">
+      <c r="J22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="K22" s="43"/>
+      <c r="K22" s="21"/>
       <c r="L22" s="19">
         <v>0</v>
       </c>
-      <c r="M22" s="42" t="s">
+      <c r="M22" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="N22" s="43"/>
+      <c r="N22" s="21"/>
       <c r="O22" s="10">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J16:K16"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A20:B20"/>
@@ -1706,46 +1749,11 @@
     <mergeCell ref="M22:N22"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Main functionality present. Will try to create .exe file
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results.xlsx
+++ b/rss_islandr/templates/results.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
   <si>
     <t>Soil</t>
   </si>
@@ -135,30 +135,6 @@
   </si>
   <si>
     <t>Industrial</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>2m</t>
-  </si>
-  <si>
-    <t>This is my site</t>
-  </si>
-  <si>
-    <t>Battery manufacture or recycling</t>
-  </si>
-  <si>
-    <t>Agricultural areas - Permanent crops</t>
-  </si>
-  <si>
-    <t>Toxic metals</t>
-  </si>
-  <si>
-    <t>No limit to access</t>
   </si>
 </sst>
 </file>
@@ -1120,18 +1096,14 @@
         <v>3</v>
       </c>
       <c r="B2" s="35"/>
-      <c r="C2" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2" t="s">
-        <v>41</v>
-      </c>
+      <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -1162,9 +1134,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="39"/>
-      <c r="C4" s="4" t="s">
-        <v>40</v>
-      </c>
+      <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -1203,7 +1173,7 @@
       </c>
       <c r="B6" s="35"/>
       <c r="C6" s="18" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1224,7 +1194,7 @@
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1245,7 +1215,7 @@
       </c>
       <c r="B8" s="28"/>
       <c r="C8" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1266,7 +1236,7 @@
       </c>
       <c r="B9" s="37"/>
       <c r="C9" s="5">
-        <v>0.48999999999999899</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1333,7 +1303,7 @@
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="18" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D12" s="32" t="s">
         <v>9</v>
@@ -1370,7 +1340,7 @@
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D13" s="27" t="s">
         <v>15</v>
@@ -1407,7 +1377,7 @@
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="18" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D14" s="27" t="s">
         <v>19</v>
@@ -1444,7 +1414,7 @@
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D15" s="27" t="s">
         <v>20</v>
@@ -1481,7 +1451,7 @@
       </c>
       <c r="B16" s="41"/>
       <c r="C16" s="18" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D16" s="36" t="s">
         <v>10</v>
@@ -1514,7 +1484,7 @@
       </c>
       <c r="B17" s="43"/>
       <c r="C17" s="10">
-        <v>0.44799999999999901</v>
+        <v>0</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1660,7 +1630,7 @@
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="19">
-        <v>0.109759999999999</v>
+        <v>0</v>
       </c>
       <c r="D22" s="20" t="s">
         <v>31</v>

</xml_diff>